<commit_message>
new update in sanity
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/zltUI/ZltTestData.xlsx
+++ b/src/test/resources/testdata/zltUI/ZltTestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gowthamraj\git\ZlaataNew19072026\src\test\resources\testdata\zltUI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gowthamraj\git\Zlaata04082026\src\test\resources\testdata\zltUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A487A85F-B99F-4D71-8E71-22E4C1D513C8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E71E61-786F-4D46-9DDC-000A5B79BEA3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{905F911F-FA1A-4DDD-B945-7467E9458D34}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6921" uniqueCount="771">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6955" uniqueCount="775">
   <si>
     <t>S.No</t>
   </si>
@@ -2317,9 +2317,6 @@
     <t>Verify login popup appears when guest user clicks Apply button in coupon section on cart page</t>
   </si>
   <si>
-    <t>Verify validation message appears when guest user clicks Gift Card Amount section on cart page</t>
-  </si>
-  <si>
     <t>Verify validation message appears when guest user clicks Threads on cart page</t>
   </si>
   <si>
@@ -2339,6 +2336,21 @@
   </si>
   <si>
     <t>Verify login popup appears when guest user clicks Profile icon in the Landing Page</t>
+  </si>
+  <si>
+    <t>Gift card</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_GC_01</t>
+  </si>
+  <si>
+    <t>Verify that the user is able to add a Gift Card to the cart</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_GC_01</t>
+  </si>
+  <si>
+    <t>Verify that the Login Popup is displayed when the user clicks the Notify Me when Available button on the Product Details Page.</t>
   </si>
 </sst>
 </file>
@@ -2805,7 +2817,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3047,6 +3059,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3082,9 +3098,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3888,7 +3901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75D1F84-2AD1-4552-9C1F-85B59D75CCFA}">
-  <dimension ref="A1:Z223"/>
+  <dimension ref="A1:Z225"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" bestFit="1" customWidth="1"/>
@@ -4639,18 +4652,18 @@
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="95" t="s">
+      <c r="A24" s="97" t="s">
         <v>155</v>
       </c>
-      <c r="B24" s="96"/>
-      <c r="C24" s="96"/>
-      <c r="D24" s="96"/>
-      <c r="E24" s="96"/>
-      <c r="F24" s="96"/>
-      <c r="G24" s="96"/>
-      <c r="H24" s="96"/>
-      <c r="I24" s="96"/>
-      <c r="J24" s="97"/>
+      <c r="B24" s="98"/>
+      <c r="C24" s="98"/>
+      <c r="D24" s="98"/>
+      <c r="E24" s="98"/>
+      <c r="F24" s="98"/>
+      <c r="G24" s="98"/>
+      <c r="H24" s="98"/>
+      <c r="I24" s="98"/>
+      <c r="J24" s="99"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="18">
@@ -5037,18 +5050,18 @@
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="98" t="s">
+      <c r="A37" s="100" t="s">
         <v>170</v>
       </c>
-      <c r="B37" s="99"/>
-      <c r="C37" s="99"/>
-      <c r="D37" s="99"/>
-      <c r="E37" s="99"/>
-      <c r="F37" s="99"/>
-      <c r="G37" s="99"/>
-      <c r="H37" s="99"/>
-      <c r="I37" s="99"/>
-      <c r="J37" s="100"/>
+      <c r="B37" s="101"/>
+      <c r="C37" s="101"/>
+      <c r="D37" s="101"/>
+      <c r="E37" s="101"/>
+      <c r="F37" s="101"/>
+      <c r="G37" s="101"/>
+      <c r="H37" s="101"/>
+      <c r="I37" s="101"/>
+      <c r="J37" s="102"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="10">
@@ -5723,18 +5736,18 @@
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="95" t="s">
+      <c r="A59" s="97" t="s">
         <v>234</v>
       </c>
-      <c r="B59" s="96"/>
-      <c r="C59" s="96"/>
-      <c r="D59" s="96"/>
-      <c r="E59" s="96"/>
-      <c r="F59" s="96"/>
-      <c r="G59" s="96"/>
-      <c r="H59" s="96"/>
-      <c r="I59" s="96"/>
-      <c r="J59" s="97"/>
+      <c r="B59" s="98"/>
+      <c r="C59" s="98"/>
+      <c r="D59" s="98"/>
+      <c r="E59" s="98"/>
+      <c r="F59" s="98"/>
+      <c r="G59" s="98"/>
+      <c r="H59" s="98"/>
+      <c r="I59" s="98"/>
+      <c r="J59" s="99"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="25">
@@ -6057,18 +6070,18 @@
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A70" s="98" t="s">
+      <c r="A70" s="100" t="s">
         <v>236</v>
       </c>
-      <c r="B70" s="99"/>
-      <c r="C70" s="99"/>
-      <c r="D70" s="99"/>
-      <c r="E70" s="99"/>
-      <c r="F70" s="99"/>
-      <c r="G70" s="99"/>
-      <c r="H70" s="99"/>
-      <c r="I70" s="99"/>
-      <c r="J70" s="100"/>
+      <c r="B70" s="101"/>
+      <c r="C70" s="101"/>
+      <c r="D70" s="101"/>
+      <c r="E70" s="101"/>
+      <c r="F70" s="101"/>
+      <c r="G70" s="101"/>
+      <c r="H70" s="101"/>
+      <c r="I70" s="101"/>
+      <c r="J70" s="102"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="25">
@@ -6487,18 +6500,18 @@
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A84" s="98" t="s">
+      <c r="A84" s="100" t="s">
         <v>334</v>
       </c>
-      <c r="B84" s="99"/>
-      <c r="C84" s="99"/>
-      <c r="D84" s="99"/>
-      <c r="E84" s="99"/>
-      <c r="F84" s="99"/>
-      <c r="G84" s="99"/>
-      <c r="H84" s="99"/>
-      <c r="I84" s="99"/>
-      <c r="J84" s="100"/>
+      <c r="B84" s="101"/>
+      <c r="C84" s="101"/>
+      <c r="D84" s="101"/>
+      <c r="E84" s="101"/>
+      <c r="F84" s="101"/>
+      <c r="G84" s="101"/>
+      <c r="H84" s="101"/>
+      <c r="I84" s="101"/>
+      <c r="J84" s="102"/>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="25">
@@ -7365,18 +7378,18 @@
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A112" s="101" t="s">
+      <c r="A112" s="103" t="s">
         <v>364</v>
       </c>
-      <c r="B112" s="101"/>
-      <c r="C112" s="101"/>
-      <c r="D112" s="101"/>
-      <c r="E112" s="101"/>
-      <c r="F112" s="101"/>
-      <c r="G112" s="101"/>
-      <c r="H112" s="101"/>
-      <c r="I112" s="101"/>
-      <c r="J112" s="101"/>
+      <c r="B112" s="103"/>
+      <c r="C112" s="103"/>
+      <c r="D112" s="103"/>
+      <c r="E112" s="103"/>
+      <c r="F112" s="103"/>
+      <c r="G112" s="103"/>
+      <c r="H112" s="103"/>
+      <c r="I112" s="103"/>
+      <c r="J112" s="103"/>
     </row>
     <row r="113" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A113" s="25">
@@ -7699,18 +7712,18 @@
       </c>
     </row>
     <row r="123" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A123" s="102" t="s">
+      <c r="A123" s="104" t="s">
         <v>366</v>
       </c>
-      <c r="B123" s="102"/>
-      <c r="C123" s="102"/>
-      <c r="D123" s="102"/>
-      <c r="E123" s="102"/>
-      <c r="F123" s="102"/>
-      <c r="G123" s="102"/>
-      <c r="H123" s="102"/>
-      <c r="I123" s="102"/>
-      <c r="J123" s="102"/>
+      <c r="B123" s="104"/>
+      <c r="C123" s="104"/>
+      <c r="D123" s="104"/>
+      <c r="E123" s="104"/>
+      <c r="F123" s="104"/>
+      <c r="G123" s="104"/>
+      <c r="H123" s="104"/>
+      <c r="I123" s="104"/>
+      <c r="J123" s="104"/>
     </row>
     <row r="124" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A124" s="25">
@@ -7745,18 +7758,18 @@
       </c>
     </row>
     <row r="125" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="102" t="s">
+      <c r="A125" s="104" t="s">
         <v>371</v>
       </c>
-      <c r="B125" s="102"/>
-      <c r="C125" s="102"/>
-      <c r="D125" s="102"/>
-      <c r="E125" s="102"/>
-      <c r="F125" s="102"/>
-      <c r="G125" s="102"/>
-      <c r="H125" s="102"/>
-      <c r="I125" s="102"/>
-      <c r="J125" s="102"/>
+      <c r="B125" s="104"/>
+      <c r="C125" s="104"/>
+      <c r="D125" s="104"/>
+      <c r="E125" s="104"/>
+      <c r="F125" s="104"/>
+      <c r="G125" s="104"/>
+      <c r="H125" s="104"/>
+      <c r="I125" s="104"/>
+      <c r="J125" s="104"/>
     </row>
     <row r="126" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A126" s="25">
@@ -7791,18 +7804,18 @@
       </c>
     </row>
     <row r="127" spans="1:24" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="102" t="s">
+      <c r="A127" s="104" t="s">
         <v>384</v>
       </c>
-      <c r="B127" s="102"/>
-      <c r="C127" s="102"/>
-      <c r="D127" s="102"/>
-      <c r="E127" s="102"/>
-      <c r="F127" s="102"/>
-      <c r="G127" s="102"/>
-      <c r="H127" s="102"/>
-      <c r="I127" s="102"/>
-      <c r="J127" s="102"/>
+      <c r="B127" s="104"/>
+      <c r="C127" s="104"/>
+      <c r="D127" s="104"/>
+      <c r="E127" s="104"/>
+      <c r="F127" s="104"/>
+      <c r="G127" s="104"/>
+      <c r="H127" s="104"/>
+      <c r="I127" s="104"/>
+      <c r="J127" s="104"/>
     </row>
     <row r="128" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="25">
@@ -8587,18 +8600,18 @@
       <c r="X144" s="58"/>
     </row>
     <row r="145" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A145" s="102" t="s">
+      <c r="A145" s="104" t="s">
         <v>396</v>
       </c>
-      <c r="B145" s="102"/>
-      <c r="C145" s="102"/>
-      <c r="D145" s="103"/>
-      <c r="E145" s="103"/>
-      <c r="F145" s="103"/>
-      <c r="G145" s="103"/>
-      <c r="H145" s="103"/>
-      <c r="I145" s="103"/>
-      <c r="J145" s="103"/>
+      <c r="B145" s="104"/>
+      <c r="C145" s="104"/>
+      <c r="D145" s="105"/>
+      <c r="E145" s="105"/>
+      <c r="F145" s="105"/>
+      <c r="G145" s="105"/>
+      <c r="H145" s="105"/>
+      <c r="I145" s="105"/>
+      <c r="J145" s="105"/>
     </row>
     <row r="146" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="59">
@@ -9061,18 +9074,18 @@
       <c r="X155" s="58"/>
     </row>
     <row r="156" spans="1:24" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A156" s="104" t="s">
+      <c r="A156" s="106" t="s">
         <v>425</v>
       </c>
-      <c r="B156" s="105"/>
-      <c r="C156" s="105"/>
-      <c r="D156" s="105"/>
-      <c r="E156" s="105"/>
-      <c r="F156" s="105"/>
-      <c r="G156" s="105"/>
-      <c r="H156" s="105"/>
-      <c r="I156" s="105"/>
-      <c r="J156" s="106"/>
+      <c r="B156" s="107"/>
+      <c r="C156" s="107"/>
+      <c r="D156" s="107"/>
+      <c r="E156" s="107"/>
+      <c r="F156" s="107"/>
+      <c r="G156" s="107"/>
+      <c r="H156" s="107"/>
+      <c r="I156" s="107"/>
+      <c r="J156" s="108"/>
     </row>
     <row r="157" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A157" s="25">
@@ -9659,18 +9672,18 @@
       <c r="X169" s="58"/>
     </row>
     <row r="170" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A170" s="102" t="s">
+      <c r="A170" s="104" t="s">
         <v>497</v>
       </c>
-      <c r="B170" s="102"/>
-      <c r="C170" s="102"/>
-      <c r="D170" s="102"/>
-      <c r="E170" s="102"/>
-      <c r="F170" s="102"/>
-      <c r="G170" s="102"/>
-      <c r="H170" s="102"/>
-      <c r="I170" s="102"/>
-      <c r="J170" s="102"/>
+      <c r="B170" s="104"/>
+      <c r="C170" s="104"/>
+      <c r="D170" s="104"/>
+      <c r="E170" s="104"/>
+      <c r="F170" s="104"/>
+      <c r="G170" s="104"/>
+      <c r="H170" s="104"/>
+      <c r="I170" s="104"/>
+      <c r="J170" s="104"/>
     </row>
     <row r="171" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A171" s="25">
@@ -9737,18 +9750,18 @@
       </c>
     </row>
     <row r="173" spans="1:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A173" s="102" t="s">
+      <c r="A173" s="104" t="s">
         <v>523</v>
       </c>
-      <c r="B173" s="102"/>
-      <c r="C173" s="102"/>
-      <c r="D173" s="102"/>
-      <c r="E173" s="102"/>
-      <c r="F173" s="102"/>
-      <c r="G173" s="102"/>
-      <c r="H173" s="102"/>
-      <c r="I173" s="102"/>
-      <c r="J173" s="102"/>
+      <c r="B173" s="104"/>
+      <c r="C173" s="104"/>
+      <c r="D173" s="104"/>
+      <c r="E173" s="104"/>
+      <c r="F173" s="104"/>
+      <c r="G173" s="104"/>
+      <c r="H173" s="104"/>
+      <c r="I173" s="104"/>
+      <c r="J173" s="104"/>
     </row>
     <row r="174" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A174" s="65">
@@ -10615,18 +10628,18 @@
       <c r="Z191" s="58"/>
     </row>
     <row r="192" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A192" s="102" t="s">
+      <c r="A192" s="104" t="s">
         <v>602</v>
       </c>
-      <c r="B192" s="102"/>
-      <c r="C192" s="102"/>
-      <c r="D192" s="102"/>
-      <c r="E192" s="102"/>
-      <c r="F192" s="102"/>
-      <c r="G192" s="102"/>
-      <c r="H192" s="102"/>
-      <c r="I192" s="102"/>
-      <c r="J192" s="102"/>
+      <c r="B192" s="104"/>
+      <c r="C192" s="104"/>
+      <c r="D192" s="104"/>
+      <c r="E192" s="104"/>
+      <c r="F192" s="104"/>
+      <c r="G192" s="104"/>
+      <c r="H192" s="104"/>
+      <c r="I192" s="104"/>
+      <c r="J192" s="104"/>
     </row>
     <row r="193" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A193" s="73">
@@ -10853,18 +10866,18 @@
       </c>
     </row>
     <row r="200" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A200" s="102" t="s">
+      <c r="A200" s="104" t="s">
         <v>602</v>
       </c>
-      <c r="B200" s="102"/>
-      <c r="C200" s="102"/>
-      <c r="D200" s="102"/>
-      <c r="E200" s="102"/>
-      <c r="F200" s="102"/>
-      <c r="G200" s="102"/>
-      <c r="H200" s="102"/>
-      <c r="I200" s="102"/>
-      <c r="J200" s="102"/>
+      <c r="B200" s="104"/>
+      <c r="C200" s="104"/>
+      <c r="D200" s="104"/>
+      <c r="E200" s="104"/>
+      <c r="F200" s="104"/>
+      <c r="G200" s="104"/>
+      <c r="H200" s="104"/>
+      <c r="I200" s="104"/>
+      <c r="J200" s="104"/>
     </row>
     <row r="201" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A201" s="73">
@@ -10899,18 +10912,18 @@
       </c>
     </row>
     <row r="202" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A202" s="107" t="s">
+      <c r="A202" s="96" t="s">
         <v>665</v>
       </c>
-      <c r="B202" s="107"/>
-      <c r="C202" s="107"/>
-      <c r="D202" s="107"/>
-      <c r="E202" s="107"/>
-      <c r="F202" s="107"/>
-      <c r="G202" s="107"/>
-      <c r="H202" s="107"/>
-      <c r="I202" s="107"/>
-      <c r="J202" s="107"/>
+      <c r="B202" s="96"/>
+      <c r="C202" s="96"/>
+      <c r="D202" s="96"/>
+      <c r="E202" s="96"/>
+      <c r="F202" s="96"/>
+      <c r="G202" s="96"/>
+      <c r="H202" s="96"/>
+      <c r="I202" s="96"/>
+      <c r="J202" s="96"/>
     </row>
     <row r="203" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A203" s="88">
@@ -11137,18 +11150,18 @@
       </c>
     </row>
     <row r="210" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A210" s="107" t="s">
+      <c r="A210" s="96" t="s">
         <v>731</v>
       </c>
-      <c r="B210" s="107"/>
-      <c r="C210" s="107"/>
-      <c r="D210" s="107"/>
-      <c r="E210" s="107"/>
-      <c r="F210" s="107"/>
-      <c r="G210" s="107"/>
-      <c r="H210" s="107"/>
-      <c r="I210" s="107"/>
-      <c r="J210" s="107"/>
+      <c r="B210" s="96"/>
+      <c r="C210" s="96"/>
+      <c r="D210" s="96"/>
+      <c r="E210" s="96"/>
+      <c r="F210" s="96"/>
+      <c r="G210" s="96"/>
+      <c r="H210" s="96"/>
+      <c r="I210" s="96"/>
+      <c r="J210" s="96"/>
     </row>
     <row r="211" spans="1:10" s="92" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A211" s="91">
@@ -11158,16 +11171,16 @@
         <v>10</v>
       </c>
       <c r="C211" s="89" t="s">
+        <v>768</v>
+      </c>
+      <c r="D211" s="94" t="s">
         <v>769</v>
-      </c>
-      <c r="D211" s="94" t="s">
-        <v>770</v>
       </c>
       <c r="E211" s="51" t="s">
         <v>14</v>
       </c>
       <c r="F211" s="89" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="G211" s="51" t="s">
         <v>11</v>
@@ -11417,7 +11430,7 @@
         <v>752</v>
       </c>
       <c r="D219" s="45" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E219" s="51" t="s">
         <v>14</v>
@@ -11449,7 +11462,7 @@
         <v>753</v>
       </c>
       <c r="D220" s="45" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="E220" s="51" t="s">
         <v>14</v>
@@ -11481,7 +11494,7 @@
         <v>754</v>
       </c>
       <c r="D221" s="45" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="E221" s="51" t="s">
         <v>14</v>
@@ -11513,7 +11526,7 @@
         <v>755</v>
       </c>
       <c r="D222" s="45" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="E222" s="51" t="s">
         <v>14</v>
@@ -11534,7 +11547,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A223" s="91">
         <v>13</v>
       </c>
@@ -11545,7 +11558,7 @@
         <v>756</v>
       </c>
       <c r="D223" s="45" t="s">
-        <v>763</v>
+        <v>774</v>
       </c>
       <c r="E223" s="51" t="s">
         <v>14</v>
@@ -11566,13 +11579,62 @@
         <v>13</v>
       </c>
     </row>
+    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A224" s="96" t="s">
+        <v>770</v>
+      </c>
+      <c r="B224" s="96"/>
+      <c r="C224" s="96"/>
+      <c r="D224" s="96"/>
+      <c r="E224" s="96"/>
+      <c r="F224" s="96"/>
+      <c r="G224" s="96"/>
+      <c r="H224" s="96"/>
+      <c r="I224" s="96"/>
+      <c r="J224" s="96"/>
+    </row>
+    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A225" s="28">
+        <v>1</v>
+      </c>
+      <c r="B225" s="86" t="s">
+        <v>10</v>
+      </c>
+      <c r="C225" s="87" t="s">
+        <v>771</v>
+      </c>
+      <c r="D225" s="95" t="s">
+        <v>772</v>
+      </c>
+      <c r="E225" s="86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F225" s="87" t="s">
+        <v>773</v>
+      </c>
+      <c r="G225" s="86" t="s">
+        <v>11</v>
+      </c>
+      <c r="H225" s="86" t="s">
+        <v>636</v>
+      </c>
+      <c r="I225" s="86" t="s">
+        <v>12</v>
+      </c>
+      <c r="J225" s="86" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A210:J210"/>
-    <mergeCell ref="A202:J202"/>
-    <mergeCell ref="A127:J127"/>
+  <mergeCells count="18">
     <mergeCell ref="A125:J125"/>
     <mergeCell ref="A123:J123"/>
+    <mergeCell ref="A224:J224"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A37:J37"/>
+    <mergeCell ref="A59:J59"/>
+    <mergeCell ref="A70:J70"/>
+    <mergeCell ref="A84:J84"/>
     <mergeCell ref="A112:J112"/>
     <mergeCell ref="A200:J200"/>
     <mergeCell ref="A192:J192"/>
@@ -11580,11 +11642,9 @@
     <mergeCell ref="A170:J170"/>
     <mergeCell ref="A145:J145"/>
     <mergeCell ref="A156:J156"/>
-    <mergeCell ref="A24:J24"/>
-    <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A59:J59"/>
-    <mergeCell ref="A70:J70"/>
-    <mergeCell ref="A84:J84"/>
+    <mergeCell ref="A210:J210"/>
+    <mergeCell ref="A202:J202"/>
+    <mergeCell ref="A127:J127"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <conditionalFormatting sqref="E2:J2 E8:J21 E23:J23">
@@ -11682,7 +11742,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE74813B-34A6-48F5-8B35-1C10409ED694}">
-  <dimension ref="A1:X216"/>
+  <dimension ref="A1:X217"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
@@ -26459,7 +26519,7 @@
     </row>
     <row r="204" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A204" s="89" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B204" s="48" t="s">
         <v>22</v>
@@ -27416,6 +27476,80 @@
         <v>22</v>
       </c>
       <c r="X216" s="48" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="217" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A217" s="87" t="s">
+        <v>773</v>
+      </c>
+      <c r="B217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="C217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="D217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="E217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="F217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="G217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="H217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="I217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="J217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="K217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="L217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="M217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="N217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="O217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="P217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="R217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="S217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="T217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="U217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="V217" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="W217" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="X217" s="48" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>